<commit_message>
QLDA: fix UC22 notification cast and template-driven Excel exports
NguoiTrinhId is bigint in DB — map as long so CoreMessaging SP runs after approve.
Resolve entity type display by const value; keep PrintTemplates as layout SOT via HandMaintainedTemplate.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/DanhSachQuanLyPheDuyet.xlsx
+++ b/QLDA.WebApi/PrintTemplates/DanhSachQuanLyPheDuyet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEFE4E52-37FB-492C-9196-039AC3375A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF949F03-EA6B-4E5C-85E4-7AAF39CB7D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -150,28 +150,28 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,92 +479,92 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="36.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="28.6640625" style="3" customWidth="1"/>
-    <col min="5" max="6" width="24.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="3"/>
+    <col min="1" max="1" width="8.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="24.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
     </row>
     <row r="3" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="6" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QLDA: feat - export Quản lý phê duyệt: tệp đính kèm, contract attachment và thứ tự cột khớp UI
- Map TepDinhKem qua PheDuyetExportMappings; export dùng IncludeAttachments=true
- DanhSachTepDinhKem luôn non-null []; AttachTepDinhKem in-memory sau ToList()
- Đổi thứ tự cột Giai đoạn / Tên bước trong template và descriptor khớp màn hình
- Template 8 cột, descriptor catalog, tests và docs v1.4

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/DanhSachQuanLyPheDuyet.xlsx
+++ b/QLDA.WebApi/PrintTemplates/DanhSachQuanLyPheDuyet.xlsx
@@ -1,116 +1,52 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF949F03-EA6B-4E5C-85E4-7AAF39CB7D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="2" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
-TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
-  </si>
-  <si>
-    <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
-Độc lập - Tự do - Hạnh phúc
----------------</t>
-  </si>
-  <si>
-    <t>DANH SÁCH PHÊ DUYỆT</t>
-  </si>
-  <si>
-    <t>STT</t>
-  </si>
-  <si>
-    <t>Dự án</t>
-  </si>
-  <si>
-    <t>Giai đoạn</t>
-  </si>
-  <si>
-    <t>Tên bước</t>
-  </si>
-  <si>
-    <t>Người trình</t>
-  </si>
-  <si>
-    <t>Người duyệt</t>
-  </si>
-  <si>
-    <t>Trạng thái</t>
-  </si>
-  <si>
-    <t>$Stt</t>
-  </si>
-  <si>
-    <t>$TenDuAn</t>
-  </si>
-  <si>
-    <t>$TenGiaiDoan</t>
-  </si>
-  <si>
-    <t>$TenBuoc</t>
-  </si>
-  <si>
-    <t>$NguoiTrinh</t>
-  </si>
-  <si>
-    <t>$NguoiDuyet</t>
-  </si>
-  <si>
-    <t>$TenTrangThai</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -146,48 +82,110 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -475,104 +473,136 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="36.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.6640625" style="1" customWidth="1"/>
-    <col min="5" max="6" width="24.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="1"/>
+    <col width="8.6640625" customWidth="1" style="1" min="1" max="1"/>
+    <col width="36.6640625" customWidth="1" style="1" min="2" max="2"/>
+    <col width="28.6640625" customWidth="1" style="1" min="3" max="3"/>
+    <col width="24.6640625" customWidth="1" style="1" min="4" max="4"/>
+    <col width="24.6640625" customWidth="1" style="1" min="5" max="6"/>
+    <col width="18.6640625" customWidth="1" style="1" min="7" max="7"/>
+    <col width="32.6640625" customWidth="1" style="1" min="8" max="8"/>
+    <col width="9.109375" customWidth="1" style="1" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
+TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
+Độc lập - Tự do - Hạnh phúc
+---------------</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
+    <row r="2"/>
+    <row r="3" ht="28.05" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>DANH SÁCH PHÊ DUYỆT</t>
+        </is>
+      </c>
     </row>
-    <row r="3" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Dự án</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Tên bước</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Người trình</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Người duyệt</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Tệp đính kèm</t>
+        </is>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>16</v>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>$Stt</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>$TenDuAn</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>$TenGiaiDoan</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>$TenBuoc</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>$NguoiTrinh</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>$NguoiDuyet</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>$TenTrangThai</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>$TepDinhKem</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="E1:H2"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A1:D2"/>
-    <mergeCell ref="E1:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>

</xml_diff>